<commit_message>
Final Version used 2024/25
</commit_message>
<xml_diff>
--- a/preise.xlsx
+++ b/preise.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ivan\Workspace\bg-school-certificate-generator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\bg-school-certificate-generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA535B3-DE50-42FB-B983-A802547D30DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2825748B-668C-4ADA-ABDF-A4D143B236D6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Konfiguration" sheetId="3" r:id="rId1"/>
@@ -399,12 +399,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86CE60E8-AF1D-4A2A-987F-130640E02E75}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.5546875" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -412,7 +412,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -420,7 +420,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -436,14 +436,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.21875" customWidth="1"/>
-    <col min="2" max="2" width="23.88671875" customWidth="1"/>
-    <col min="3" max="3" width="16.109375" customWidth="1"/>
+    <col min="1" max="1" width="22.28515625" customWidth="1"/>
+    <col min="2" max="2" width="23.85546875" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -451,7 +451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -459,15 +459,15 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
     </row>
@@ -480,9 +480,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A74978CF-B58C-4F9A-B63A-B7C10EF99CCA}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -490,23 +490,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="2">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -530,6 +530,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="69b70055-4ccd-41e5-ba44-04aa7b40ef87">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="0d7d4427-3d9a-4210-88a6-80411ae356c7" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100202D4B9E3A436A44B91CC234F5A1B18B" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="faa7d1780a64debc3e5433f1993c437a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="69b70055-4ccd-41e5-ba44-04aa7b40ef87" xmlns:ns3="0d7d4427-3d9a-4210-88a6-80411ae356c7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="46ac9b7ec201ca2a68a6a1e758789984" ns2:_="" ns3:_="">
     <xsd:import namespace="69b70055-4ccd-41e5-ba44-04aa7b40ef87"/>
@@ -724,17 +735,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="69b70055-4ccd-41e5-ba44-04aa7b40ef87">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="0d7d4427-3d9a-4210-88a6-80411ae356c7" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A75E2A0C-A03D-4EF1-AA2F-BC86D3F36961}">
   <ds:schemaRefs>
@@ -744,6 +744,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6E074D9-8A3F-4B12-8FF2-84C884A0412A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="69b70055-4ccd-41e5-ba44-04aa7b40ef87"/>
+    <ds:schemaRef ds:uri="0d7d4427-3d9a-4210-88a6-80411ae356c7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98CB3CB1-47E5-4ECC-B8C0-D8BE43DCE475}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -760,15 +771,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6E074D9-8A3F-4B12-8FF2-84C884A0412A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="69b70055-4ccd-41e5-ba44-04aa7b40ef87"/>
-    <ds:schemaRef ds:uri="0d7d4427-3d9a-4210-88a6-80411ae356c7"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>